<commit_message>
Finalised Excel model and prepared for Power BI
</commit_message>
<xml_diff>
--- a/data/construction_cost_dashboard.xlsx.xlsx
+++ b/data/construction_cost_dashboard.xlsx.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\qs\construction-cost-dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5295A69-5166-4FB3-9A46-97EF3BA7459A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7785AFD0-C475-4448-8A63-7B7F26A8C4DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="2355" windowWidth="29040" windowHeight="16440" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_BoQ" sheetId="1" r:id="rId1"/>
@@ -213,8 +213,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="167" formatCode="&quot;£&quot;#,##0.00"/>
-    <numFmt numFmtId="170" formatCode="&quot;£&quot;#,##0"/>
+    <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;£&quot;#,##0"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -253,8 +253,8 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -262,30 +262,48 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="17">
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;£&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;£&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;£&quot;#,##0.00"/>
+      <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;£&quot;#,##0.00"/>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;£&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
@@ -295,21 +313,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;£&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="170" formatCode="&quot;£&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="170" formatCode="&quot;£&quot;#,##0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -325,39 +328,39 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0C6C3F10-0AEF-407A-B71B-D62A935FC0A4}" name="Table1" displayName="Table1" ref="A1:D13" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0C6C3F10-0AEF-407A-B71B-D62A935FC0A4}" name="tbl_boq" displayName="tbl_boq" ref="A1:D13" totalsRowShown="0">
   <autoFilter ref="A1:D13" xr:uid="{0C6C3F10-0AEF-407A-B71B-D62A935FC0A4}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{A54D2983-44D5-4CC4-8F53-C763ABFA2C90}" name="Item_ID"/>
     <tableColumn id="2" xr3:uid="{43E72617-AE41-4AD8-8DEC-0D0F6C63B3C6}" name="Work_Package"/>
     <tableColumn id="3" xr3:uid="{1FBF5717-4BAD-4B88-B54E-E694A0784D3D}" name="Category"/>
-    <tableColumn id="4" xr3:uid="{BC438E18-83FA-4305-8A49-8F98AC445249}" name="Budget_GBP" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{BC438E18-83FA-4305-8A49-8F98AC445249}" name="Budget_GBP" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{18CAA750-DD71-4F52-BB96-2081A97B6D56}" name="Table2" displayName="Table2" ref="A1:C21" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{18CAA750-DD71-4F52-BB96-2081A97B6D56}" name="tbl_monthly_cost" displayName="tbl_monthly_cost" ref="A1:C21" totalsRowShown="0">
   <autoFilter ref="A1:C21" xr:uid="{18CAA750-DD71-4F52-BB96-2081A97B6D56}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{2000578B-6209-4150-A755-A656196B0F48}" name="Month"/>
+    <tableColumn id="1" xr3:uid="{2000578B-6209-4150-A755-A656196B0F48}" name="Month" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{90F3E908-129A-4239-9B48-259E1332327D}" name="Category"/>
-    <tableColumn id="3" xr3:uid="{772AF29B-F73E-418D-A681-28EB4B8551FE}" name="Actual_Cost_GBP" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{772AF29B-F73E-418D-A681-28EB4B8551FE}" name="Actual_Cost_GBP" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{E42225C4-8FF6-49B5-AB3A-2EB457E9E866}" name="Table6" displayName="Table6" ref="A1:C13" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{E42225C4-8FF6-49B5-AB3A-2EB457E9E866}" name="tbl_monthly_summary" displayName="tbl_monthly_summary" ref="A1:C13" totalsRowShown="0">
   <autoFilter ref="A1:C13" xr:uid="{E42225C4-8FF6-49B5-AB3A-2EB457E9E866}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{1388AA3A-5BAA-4A45-9ACC-8B5D2B281B77}" name="Month" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{2B156260-0DD9-4851-9ECA-B25D1A3EB95F}" name="Monthly_Total_GBP" dataDxfId="4">
+    <tableColumn id="1" xr3:uid="{1388AA3A-5BAA-4A45-9ACC-8B5D2B281B77}" name="Month" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{2B156260-0DD9-4851-9ECA-B25D1A3EB95F}" name="Monthly_Total_GBP" dataDxfId="1">
       <calculatedColumnFormula>SUMIFS('02_Monthly_Costs'!C:C, '02_Monthly_Costs'!A:A, A2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{7A8FD010-5122-44F5-A21D-5F005DDC100E}" name="Cumulative_AC_GBP" dataDxfId="3">
+    <tableColumn id="3" xr3:uid="{7A8FD010-5122-44F5-A21D-5F005DDC100E}" name="Cumulative_AC_GBP" dataDxfId="0">
       <calculatedColumnFormula>B1</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -366,10 +369,10 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E43BCDD9-CDD9-4C9C-B94E-CB324866C5BA}" name="Table3" displayName="Table3" ref="A1:C13" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E43BCDD9-CDD9-4C9C-B94E-CB324866C5BA}" name="tbl_progress" displayName="tbl_progress" ref="A1:C13" totalsRowShown="0">
   <autoFilter ref="A1:C13" xr:uid="{E43BCDD9-CDD9-4C9C-B94E-CB324866C5BA}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{3901290D-1847-467A-B043-6CCF42EBAF4A}" name="Month" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{3901290D-1847-467A-B043-6CCF42EBAF4A}" name="Month" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{FEA6880E-02FF-4AAB-AAB0-95A267F2B868}" name="Planned_Progress_Pct"/>
     <tableColumn id="3" xr3:uid="{3684B450-3A0B-4362-BEE4-CE03E9609A99}" name="Actual_Progress_Pct"/>
   </tableColumns>
@@ -378,7 +381,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{85B0BEA2-22C4-4A68-B563-C1D1AE0B5BF3}" name="Table4" displayName="Table4" ref="A1:B6" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{85B0BEA2-22C4-4A68-B563-C1D1AE0B5BF3}" name="tbl_project_info" displayName="tbl_project_info" ref="A1:B6" totalsRowShown="0">
   <autoFilter ref="A1:B6" xr:uid="{85B0BEA2-22C4-4A68-B563-C1D1AE0B5BF3}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{030DFBC1-976C-4393-B2C5-53FB80EBCFE8}" name="Field"/>
@@ -389,36 +392,36 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1E3B767B-F2B1-4FBD-BEB7-8A6DCE7ECDDF}" name="EVM_Table" displayName="EVM_Table" ref="A1:J13" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1E3B767B-F2B1-4FBD-BEB7-8A6DCE7ECDDF}" name="tbl_evm" displayName="tbl_evm" ref="A1:J13" totalsRowShown="0">
   <autoFilter ref="A1:J13" xr:uid="{1E3B767B-F2B1-4FBD-BEB7-8A6DCE7ECDDF}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{D334BF16-892B-40A6-AD22-76E25F45C9F4}" name="Month" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{4E438E52-2DAD-4B51-87A1-4E35F4A63EB6}" name="Planned_Progress_Pct" dataDxfId="9">
+    <tableColumn id="1" xr3:uid="{D334BF16-892B-40A6-AD22-76E25F45C9F4}" name="Month" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{4E438E52-2DAD-4B51-87A1-4E35F4A63EB6}" name="Planned_Progress_Pct" dataDxfId="15">
       <calculatedColumnFormula>'03_Progress'!B2*0.01</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{6B330E2A-268A-4F93-B932-CFAD88BF7CE4}" name="Actual_Progress_Pct" dataDxfId="8">
+    <tableColumn id="3" xr3:uid="{6B330E2A-268A-4F93-B932-CFAD88BF7CE4}" name="Actual_Progress_Pct" dataDxfId="14">
       <calculatedColumnFormula>'03_Progress'!C2*0.01</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{1B182485-FC7B-45B4-8316-DF0A88E44868}" name="PV_GBP" dataDxfId="7">
-      <calculatedColumnFormula>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Planned_Progress_Pct]]</calculatedColumnFormula>
+    <tableColumn id="4" xr3:uid="{1B182485-FC7B-45B4-8316-DF0A88E44868}" name="PV_GBP" dataDxfId="13">
+      <calculatedColumnFormula>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Planned_Progress_Pct]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{B41AB69F-C8C1-4FEE-B902-920159776DD0}" name="EV_GBP" dataDxfId="6">
-      <calculatedColumnFormula>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Actual_Progress_Pct]]</calculatedColumnFormula>
+    <tableColumn id="5" xr3:uid="{B41AB69F-C8C1-4FEE-B902-920159776DD0}" name="EV_GBP" dataDxfId="12">
+      <calculatedColumnFormula>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Actual_Progress_Pct]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A56094F4-2E91-410E-A6ED-E75E4B823C94}" name="AC_GBP" dataDxfId="12">
+    <tableColumn id="6" xr3:uid="{A56094F4-2E91-410E-A6ED-E75E4B823C94}" name="AC_GBP" dataDxfId="11">
       <calculatedColumnFormula>'02B_Monthly_Summary'!C2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{7807CCDD-DE13-44B2-B542-076FBFD8AA1D}" name="CV_GBP" dataDxfId="2">
-      <calculatedColumnFormula>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[AC_GBP]]</calculatedColumnFormula>
+    <tableColumn id="7" xr3:uid="{7807CCDD-DE13-44B2-B542-076FBFD8AA1D}" name="CV_GBP" dataDxfId="10">
+      <calculatedColumnFormula>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[AC_GBP]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B3B19D80-8CA9-4B5D-AB72-6318BCB79355}" name="SV_GBP" dataDxfId="1">
-      <calculatedColumnFormula>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[PV_GBP]]</calculatedColumnFormula>
+    <tableColumn id="8" xr3:uid="{B3B19D80-8CA9-4B5D-AB72-6318BCB79355}" name="SV_GBP" dataDxfId="9">
+      <calculatedColumnFormula>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[PV_GBP]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{9D54921C-9196-4478-AEF2-2B322EA08379}" name="CPI" dataDxfId="0">
-      <calculatedColumnFormula>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[AC_GBP]]</calculatedColumnFormula>
+    <tableColumn id="9" xr3:uid="{9D54921C-9196-4478-AEF2-2B322EA08379}" name="CPI" dataDxfId="8">
+      <calculatedColumnFormula>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[AC_GBP]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{F0706BE6-520A-4731-A219-8AF3C30AAE6D}" name="SPI" dataDxfId="11">
-      <calculatedColumnFormula>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[PV_GBP]]</calculatedColumnFormula>
+    <tableColumn id="10" xr3:uid="{F0706BE6-520A-4731-A219-8AF3C30AAE6D}" name="SPI" dataDxfId="7">
+      <calculatedColumnFormula>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[PV_GBP]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -889,7 +892,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{515F7D25-61BB-4AEE-817E-1E60260F3F57}">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="8.3828125" customWidth="1"/>
@@ -897,235 +900,238 @@
     <col min="3" max="3" width="17.15234375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>22</v>
       </c>
       <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A2" s="4" t="s">
         <v>24</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2">
-        <v>180000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+      <c r="C2" s="1">
+        <v>288000</v>
+      </c>
+      <c r="K2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A3" s="4" t="s">
         <v>25</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="2">
-        <v>260000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
+      <c r="C3" s="1">
+        <v>416000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A4" s="4" t="s">
         <v>26</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="2">
-        <v>210000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
+      <c r="C4" s="1">
+        <v>336000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A5" s="4" t="s">
         <v>26</v>
       </c>
       <c r="B5" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="2">
-        <v>300000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
+      <c r="C5" s="1">
+        <v>480000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A6" s="4" t="s">
         <v>27</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="2">
-        <v>520000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
+      <c r="C6" s="1">
+        <v>832000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A7" s="4" t="s">
         <v>28</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="2">
-        <v>610000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
+      <c r="C7" s="1">
+        <v>976000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A8" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B8" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="2">
-        <v>700000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
+      <c r="C8" s="1">
+        <v>1120000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A9" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B9" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="2">
-        <v>180000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
+      <c r="C9" s="1">
+        <v>288000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A10" s="4" t="s">
         <v>30</v>
       </c>
       <c r="B10" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="2">
-        <v>260000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
+      <c r="C10" s="1">
+        <v>416000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A11" s="4" t="s">
         <v>30</v>
       </c>
       <c r="B11" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="2">
-        <v>220000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
+      <c r="C11" s="1">
+        <v>352000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A12" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B12" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="2">
-        <v>240000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
+      <c r="C12" s="1">
+        <v>384000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A13" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B13" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="2">
-        <v>340000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A14" t="s">
+      <c r="C13" s="1">
+        <v>544000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A14" s="4" t="s">
         <v>32</v>
       </c>
       <c r="B14" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="2">
-        <v>420000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A15" t="s">
+      <c r="C14" s="1">
+        <v>672000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A15" s="4" t="s">
         <v>32</v>
       </c>
       <c r="B15" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="2">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A16" t="s">
+      <c r="C15" s="1">
+        <v>240000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A16" s="4" t="s">
         <v>33</v>
       </c>
       <c r="B16" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="2">
-        <v>380000</v>
+      <c r="C16" s="1">
+        <v>608000</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A17" t="s">
+      <c r="A17" s="4" t="s">
         <v>33</v>
       </c>
       <c r="B17" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="2">
-        <v>220000</v>
+      <c r="C17" s="1">
+        <v>352000</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A18" t="s">
+      <c r="A18" s="4" t="s">
         <v>34</v>
       </c>
       <c r="B18" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="2">
-        <v>260000</v>
+      <c r="C18" s="1">
+        <v>416000</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A19" t="s">
+      <c r="A19" s="4" t="s">
         <v>34</v>
       </c>
       <c r="B19" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="2">
-        <v>120000</v>
+      <c r="C19" s="1">
+        <v>192000</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A20" t="s">
+      <c r="A20" s="4" t="s">
         <v>35</v>
       </c>
       <c r="B20" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="2">
-        <v>180000</v>
+      <c r="C20" s="1">
+        <v>288000</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A21" t="s">
+      <c r="A21" s="4" t="s">
         <v>35</v>
       </c>
       <c r="B21" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="2">
-        <v>160000</v>
+      <c r="C21" s="1">
+        <v>256000</v>
       </c>
     </row>
   </sheetData>
@@ -1161,156 +1167,156 @@
       <c r="A2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <f>SUMIFS('02_Monthly_Costs'!C:C, '02_Monthly_Costs'!A:A, A2)</f>
-        <v>180000</v>
-      </c>
-      <c r="C2">
+        <v>288000</v>
+      </c>
+      <c r="C2" s="1">
         <f>B2</f>
-        <v>180000</v>
+        <v>288000</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <f>SUMIFS('02_Monthly_Costs'!C:C, '02_Monthly_Costs'!A:A, A3)</f>
-        <v>260000</v>
-      </c>
-      <c r="C3">
-        <f>C2+Table6[[#This Row],[Monthly_Total_GBP]]</f>
-        <v>440000</v>
+        <v>416000</v>
+      </c>
+      <c r="C3" s="1">
+        <f>C2+tbl_monthly_summary[[#This Row],[Monthly_Total_GBP]]</f>
+        <v>704000</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <f>SUMIFS('02_Monthly_Costs'!C:C, '02_Monthly_Costs'!A:A, A4)</f>
-        <v>510000</v>
-      </c>
-      <c r="C4">
-        <f>C3+Table6[[#This Row],[Monthly_Total_GBP]]</f>
-        <v>950000</v>
+        <v>816000</v>
+      </c>
+      <c r="C4" s="1">
+        <f>C3+tbl_monthly_summary[[#This Row],[Monthly_Total_GBP]]</f>
+        <v>1520000</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="1">
         <f>SUMIFS('02_Monthly_Costs'!C:C, '02_Monthly_Costs'!A:A, A5)</f>
-        <v>520000</v>
-      </c>
-      <c r="C5">
-        <f>C4+Table6[[#This Row],[Monthly_Total_GBP]]</f>
-        <v>1470000</v>
+        <v>832000</v>
+      </c>
+      <c r="C5" s="1">
+        <f>C4+tbl_monthly_summary[[#This Row],[Monthly_Total_GBP]]</f>
+        <v>2352000</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="1">
         <f>SUMIFS('02_Monthly_Costs'!C:C, '02_Monthly_Costs'!A:A, A6)</f>
-        <v>610000</v>
-      </c>
-      <c r="C6">
-        <f>C5+Table6[[#This Row],[Monthly_Total_GBP]]</f>
-        <v>2080000</v>
+        <v>976000</v>
+      </c>
+      <c r="C6" s="1">
+        <f>C5+tbl_monthly_summary[[#This Row],[Monthly_Total_GBP]]</f>
+        <v>3328000</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="1">
         <f>SUMIFS('02_Monthly_Costs'!C:C, '02_Monthly_Costs'!A:A, A7)</f>
-        <v>880000</v>
-      </c>
-      <c r="C7">
-        <f>C6+Table6[[#This Row],[Monthly_Total_GBP]]</f>
-        <v>2960000</v>
+        <v>1408000</v>
+      </c>
+      <c r="C7" s="1">
+        <f>C6+tbl_monthly_summary[[#This Row],[Monthly_Total_GBP]]</f>
+        <v>4736000</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="1">
         <f>SUMIFS('02_Monthly_Costs'!C:C, '02_Monthly_Costs'!A:A, A8)</f>
-        <v>480000</v>
-      </c>
-      <c r="C8">
-        <f>C7+Table6[[#This Row],[Monthly_Total_GBP]]</f>
-        <v>3440000</v>
+        <v>768000</v>
+      </c>
+      <c r="C8" s="1">
+        <f>C7+tbl_monthly_summary[[#This Row],[Monthly_Total_GBP]]</f>
+        <v>5504000</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="1">
         <f>SUMIFS('02_Monthly_Costs'!C:C, '02_Monthly_Costs'!A:A, A9)</f>
-        <v>580000</v>
-      </c>
-      <c r="C9">
-        <f>C8+Table6[[#This Row],[Monthly_Total_GBP]]</f>
-        <v>4020000</v>
+        <v>928000</v>
+      </c>
+      <c r="C9" s="1">
+        <f>C8+tbl_monthly_summary[[#This Row],[Monthly_Total_GBP]]</f>
+        <v>6432000</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="1">
         <f>SUMIFS('02_Monthly_Costs'!C:C, '02_Monthly_Costs'!A:A, A10)</f>
-        <v>570000</v>
-      </c>
-      <c r="C10">
-        <f>C9+Table6[[#This Row],[Monthly_Total_GBP]]</f>
-        <v>4590000</v>
+        <v>912000</v>
+      </c>
+      <c r="C10" s="1">
+        <f>C9+tbl_monthly_summary[[#This Row],[Monthly_Total_GBP]]</f>
+        <v>7344000</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="1">
         <f>SUMIFS('02_Monthly_Costs'!C:C, '02_Monthly_Costs'!A:A, A11)</f>
-        <v>600000</v>
-      </c>
-      <c r="C11">
-        <f>C10+Table6[[#This Row],[Monthly_Total_GBP]]</f>
-        <v>5190000</v>
+        <v>960000</v>
+      </c>
+      <c r="C11" s="1">
+        <f>C10+tbl_monthly_summary[[#This Row],[Monthly_Total_GBP]]</f>
+        <v>8304000</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="1">
         <f>SUMIFS('02_Monthly_Costs'!C:C, '02_Monthly_Costs'!A:A, A12)</f>
-        <v>380000</v>
-      </c>
-      <c r="C12">
-        <f>C11+Table6[[#This Row],[Monthly_Total_GBP]]</f>
-        <v>5570000</v>
+        <v>608000</v>
+      </c>
+      <c r="C12" s="1">
+        <f>C11+tbl_monthly_summary[[#This Row],[Monthly_Total_GBP]]</f>
+        <v>8912000</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="1">
         <f>SUMIFS('02_Monthly_Costs'!C:C, '02_Monthly_Costs'!A:A, A13)</f>
-        <v>340000</v>
-      </c>
-      <c r="C13">
-        <f>C12+Table6[[#This Row],[Monthly_Total_GBP]]</f>
-        <v>5910000</v>
+        <v>544000</v>
+      </c>
+      <c r="C13" s="1">
+        <f>C12+tbl_monthly_summary[[#This Row],[Monthly_Total_GBP]]</f>
+        <v>9456000</v>
       </c>
     </row>
   </sheetData>
@@ -1610,31 +1616,31 @@
         <v>0.02</v>
       </c>
       <c r="D2" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Planned_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Planned_Progress_Pct]]</f>
         <v>285000</v>
       </c>
       <c r="E2" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Actual_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Actual_Progress_Pct]]</f>
         <v>190000</v>
       </c>
       <c r="F2" s="1">
         <f>'02B_Monthly_Summary'!C2</f>
-        <v>180000</v>
+        <v>288000</v>
       </c>
       <c r="G2" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>10000</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>-98000</v>
       </c>
       <c r="H2" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>-95000</v>
       </c>
       <c r="I2" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>1.0555555555555556</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>0.65972222222222221</v>
       </c>
       <c r="J2" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>0.66666666666666663</v>
       </c>
     </row>
@@ -1651,31 +1657,31 @@
         <v>0.06</v>
       </c>
       <c r="D3" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Planned_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Planned_Progress_Pct]]</f>
         <v>760000</v>
       </c>
       <c r="E3" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Actual_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Actual_Progress_Pct]]</f>
         <v>570000</v>
       </c>
       <c r="F3" s="1">
         <f>'02B_Monthly_Summary'!C3</f>
-        <v>440000</v>
+        <v>704000</v>
       </c>
       <c r="G3" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>130000</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>-134000</v>
       </c>
       <c r="H3" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>-190000</v>
       </c>
       <c r="I3" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>1.2954545454545454</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>0.80965909090909094</v>
       </c>
       <c r="J3" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>0.75</v>
       </c>
     </row>
@@ -1692,31 +1698,31 @@
         <v>0.12</v>
       </c>
       <c r="D4" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Planned_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Planned_Progress_Pct]]</f>
         <v>1425000</v>
       </c>
       <c r="E4" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Actual_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Actual_Progress_Pct]]</f>
         <v>1140000</v>
       </c>
       <c r="F4" s="1">
         <f>'02B_Monthly_Summary'!C4</f>
-        <v>950000</v>
+        <v>1520000</v>
       </c>
       <c r="G4" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>190000</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>-380000</v>
       </c>
       <c r="H4" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>-285000</v>
       </c>
       <c r="I4" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>1.2</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>0.75</v>
       </c>
       <c r="J4" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>0.8</v>
       </c>
     </row>
@@ -1733,31 +1739,31 @@
         <v>0.2</v>
       </c>
       <c r="D5" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Planned_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Planned_Progress_Pct]]</f>
         <v>2280000</v>
       </c>
       <c r="E5" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Actual_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Actual_Progress_Pct]]</f>
         <v>1900000</v>
       </c>
       <c r="F5" s="1">
         <f>'02B_Monthly_Summary'!C5</f>
-        <v>1470000</v>
+        <v>2352000</v>
       </c>
       <c r="G5" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>430000</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>-452000</v>
       </c>
       <c r="H5" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>-380000</v>
       </c>
       <c r="I5" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>1.2925170068027212</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>0.80782312925170063</v>
       </c>
       <c r="J5" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>0.83333333333333337</v>
       </c>
     </row>
@@ -1774,31 +1780,31 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="D6" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Planned_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Planned_Progress_Pct]]</f>
         <v>3230000</v>
       </c>
       <c r="E6" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Actual_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Actual_Progress_Pct]]</f>
         <v>2755000</v>
       </c>
       <c r="F6" s="1">
         <f>'02B_Monthly_Summary'!C6</f>
-        <v>2080000</v>
+        <v>3328000</v>
       </c>
       <c r="G6" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>675000</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>-573000</v>
       </c>
       <c r="H6" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>-475000</v>
       </c>
       <c r="I6" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>1.3245192307692308</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>0.82782451923076927</v>
       </c>
       <c r="J6" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>0.8529411764705882</v>
       </c>
     </row>
@@ -1815,31 +1821,31 @@
         <v>0.4</v>
       </c>
       <c r="D7" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Planned_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Planned_Progress_Pct]]</f>
         <v>4275000</v>
       </c>
       <c r="E7" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Actual_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Actual_Progress_Pct]]</f>
         <v>3800000</v>
       </c>
       <c r="F7" s="1">
         <f>'02B_Monthly_Summary'!C7</f>
-        <v>2960000</v>
+        <v>4736000</v>
       </c>
       <c r="G7" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>840000</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>-936000</v>
       </c>
       <c r="H7" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>-475000</v>
       </c>
       <c r="I7" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>1.2837837837837838</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>0.80236486486486491</v>
       </c>
       <c r="J7" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>0.88888888888888884</v>
       </c>
     </row>
@@ -1856,31 +1862,31 @@
         <v>0.51</v>
       </c>
       <c r="D8" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Planned_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Planned_Progress_Pct]]</f>
         <v>5415000.0000000009</v>
       </c>
       <c r="E8" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Actual_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Actual_Progress_Pct]]</f>
         <v>4845000</v>
       </c>
       <c r="F8" s="1">
         <f>'02B_Monthly_Summary'!C8</f>
-        <v>3440000</v>
+        <v>5504000</v>
       </c>
       <c r="G8" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>1405000</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>-659000</v>
       </c>
       <c r="H8" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>-570000.00000000093</v>
       </c>
       <c r="I8" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>1.4084302325581395</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>0.88026889534883723</v>
       </c>
       <c r="J8" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>0.89473684210526305</v>
       </c>
     </row>
@@ -1897,31 +1903,31 @@
         <v>0.61</v>
       </c>
       <c r="D9" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Planned_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Planned_Progress_Pct]]</f>
         <v>6460000</v>
       </c>
       <c r="E9" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Actual_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Actual_Progress_Pct]]</f>
         <v>5795000</v>
       </c>
       <c r="F9" s="1">
         <f>'02B_Monthly_Summary'!C9</f>
-        <v>4020000</v>
+        <v>6432000</v>
       </c>
       <c r="G9" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>1775000</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>-637000</v>
       </c>
       <c r="H9" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>-665000</v>
       </c>
       <c r="I9" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>1.441542288557214</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>0.90096393034825872</v>
       </c>
       <c r="J9" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>0.8970588235294118</v>
       </c>
     </row>
@@ -1938,31 +1944,31 @@
         <v>0.71</v>
       </c>
       <c r="D10" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Planned_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Planned_Progress_Pct]]</f>
         <v>7410000</v>
       </c>
       <c r="E10" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Actual_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Actual_Progress_Pct]]</f>
         <v>6745000</v>
       </c>
       <c r="F10" s="1">
         <f>'02B_Monthly_Summary'!C10</f>
-        <v>4590000</v>
+        <v>7344000</v>
       </c>
       <c r="G10" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>2155000</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>-599000</v>
       </c>
       <c r="H10" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>-665000</v>
       </c>
       <c r="I10" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>1.4694989106753813</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>0.91843681917211328</v>
       </c>
       <c r="J10" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>0.91025641025641024</v>
       </c>
     </row>
@@ -1979,31 +1985,31 @@
         <v>0.81</v>
       </c>
       <c r="D11" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Planned_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Planned_Progress_Pct]]</f>
         <v>8265000</v>
       </c>
       <c r="E11" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Actual_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Actual_Progress_Pct]]</f>
         <v>7695000.0000000009</v>
       </c>
       <c r="F11" s="1">
         <f>'02B_Monthly_Summary'!C11</f>
-        <v>5190000</v>
+        <v>8304000</v>
       </c>
       <c r="G11" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>2505000.0000000009</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>-608999.99999999907</v>
       </c>
       <c r="H11" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>-569999.99999999907</v>
       </c>
       <c r="I11" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>1.4826589595375725</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>0.92666184971098275</v>
       </c>
       <c r="J11" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>0.93103448275862077</v>
       </c>
     </row>
@@ -2020,31 +2026,31 @@
         <v>0.9</v>
       </c>
       <c r="D12" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Planned_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Planned_Progress_Pct]]</f>
         <v>9025000</v>
       </c>
       <c r="E12" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Actual_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Actual_Progress_Pct]]</f>
         <v>8550000</v>
       </c>
       <c r="F12" s="1">
         <f>'02B_Monthly_Summary'!C12</f>
-        <v>5570000</v>
+        <v>8912000</v>
       </c>
       <c r="G12" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>2980000</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>-362000</v>
       </c>
       <c r="H12" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>-475000</v>
       </c>
       <c r="I12" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>1.5350089766606823</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>0.95938061041292644</v>
       </c>
       <c r="J12" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>0.94736842105263153</v>
       </c>
     </row>
@@ -2061,31 +2067,31 @@
         <v>0.96</v>
       </c>
       <c r="D13" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Planned_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Planned_Progress_Pct]]</f>
         <v>9500000</v>
       </c>
       <c r="E13" s="1">
-        <f>'04_Project_Info'!$B$3*EVM_Table[[#This Row],[Actual_Progress_Pct]]</f>
+        <f>'04_Project_Info'!$B$3*tbl_evm[[#This Row],[Actual_Progress_Pct]]</f>
         <v>9120000</v>
       </c>
       <c r="F13" s="1">
         <f>'02B_Monthly_Summary'!C13</f>
-        <v>5910000</v>
+        <v>9456000</v>
       </c>
       <c r="G13" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>3210000</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>-336000</v>
       </c>
       <c r="H13" s="1">
-        <f>EVM_Table[[#This Row],[EV_GBP]]-EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]-tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>-380000</v>
       </c>
       <c r="I13" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[AC_GBP]]</f>
-        <v>1.5431472081218274</v>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[AC_GBP]]</f>
+        <v>0.96446700507614214</v>
       </c>
       <c r="J13" s="3">
-        <f>EVM_Table[[#This Row],[EV_GBP]]/EVM_Table[[#This Row],[PV_GBP]]</f>
+        <f>tbl_evm[[#This Row],[EV_GBP]]/tbl_evm[[#This Row],[PV_GBP]]</f>
         <v>0.96</v>
       </c>
     </row>

</xml_diff>